<commit_message>
v1.12 scorer-tag corrections + add sync infrastructure
- Row 29 BUF/BOS G4: tag S. Kuraly (SH) per NHL.com recap
- Row 32 EDM/ANA G4: tag R. Nugent-Hopkins (PP), M. Granlund (PP), E. Bouchard (PP)
- Add AGENT/sync-latest.sh (local launchd job script)
- Add SESSION_LOGS/ folder with 2026-04-26 session record
</commit_message>
<xml_diff>
--- a/2026 NHL Playoffs_v1.12.xlsx
+++ b/2026 NHL Playoffs_v1.12.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1520" yWindow="1100" windowWidth="27640" windowHeight="16660" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="2026 NHL Playoffs_By Dates" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="By Series" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="By Team" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="By Division" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Bracket" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 NHL Playoffs_By Dates" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Series" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Team" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Division" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bracket" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -3173,7 +3173,7 @@
       </c>
       <c r="J29" s="65" t="inlineStr">
         <is>
-          <t>BUF: P. Krebs, J. Doan (GW), Z. Benson, B. Byram, B. Malenstyn, A. Tuch | BOS: S. Kuraly</t>
+          <t>BUF: P. Krebs, J. Doan (GW), Z. Benson, B. Byram, B. Malenstyn, A. Tuch | BOS: S. Kuraly (SH)</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="J32" s="65" t="inlineStr">
         <is>
-          <t>ANA: C. Gauthier (PP), M. Granlund, J. Viel, R. Poehling (OT winner) | EDM: K. Kapanen, E. Bouchard, R. Nugent-Hopkins</t>
+          <t>ANA: C. Gauthier (PP), M. Granlund (PP), J. Viel, R. Poehling (OT winner) | EDM: K. Kapanen, R. Nugent-Hopkins (PP), E. Bouchard (PP)</t>
         </is>
       </c>
     </row>

</xml_diff>